<commit_message>
Build capital state model and capital engine
</commit_message>
<xml_diff>
--- a/dashboard/trading_system.xlsx
+++ b/dashboard/trading_system.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\husainnatha\tradingsystem\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2063A75-E978-4C9C-B807-BB0B021E352D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4DE365-0BBE-4192-B497-17133FA8C8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="353" yWindow="1343" windowWidth="16200" windowHeight="9307" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONTRIBUTIONS" sheetId="11" r:id="rId1"/>
@@ -1000,7 +1000,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1949" uniqueCount="607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1950" uniqueCount="608">
   <si>
     <t>collected_timestamp</t>
   </si>
@@ -2925,6 +2925,9 @@
   </si>
   <si>
     <t>max_deployment_percent</t>
+  </si>
+  <si>
+    <t>Column1</t>
   </si>
 </sst>
 </file>
@@ -3068,7 +3071,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3146,11 +3149,44 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="53">
+  <dxfs count="54">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FFF0F0F0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="13" formatCode="0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF0C0E12"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FFA0A0A0"/>
@@ -9511,7 +9547,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F82495E7-9F34-4C1F-83EC-FA45D59FA2BD}" name="tblContributions" displayName="tblContributions" ref="A1:C2" totalsRowShown="0">
   <autoFilter ref="A1:C2" xr:uid="{F82495E7-9F34-4C1F-83EC-FA45D59FA2BD}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{EAE9033F-E950-4D8F-AC60-78CCDA7A0C9E}" name="DATE" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{EAE9033F-E950-4D8F-AC60-78CCDA7A0C9E}" name="DATE" dataDxfId="53"/>
     <tableColumn id="2" xr3:uid="{1D40F1FF-D66C-4703-9DEC-93C768793D8F}" name="AMMOUNT"/>
     <tableColumn id="3" xr3:uid="{49855D82-DE07-4257-837D-DD0BE41E988B}" name="Notes"/>
   </tableColumns>
@@ -9539,64 +9575,64 @@
   <tableColumns count="31">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="symbol"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="StockName"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="LastTradeTime" dataDxfId="51">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="LastTradeTime" dataDxfId="52">
       <calculatedColumnFormula array="1">_FV(B2,"Last trade time",TRUE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="TradeCurrency">
       <calculatedColumnFormula array="1">_FV(B2,"Currency")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="StockPrice" dataDxfId="50">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="StockPrice" dataDxfId="51">
       <calculatedColumnFormula array="1">_FV(B2,"Price")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ChangePercent" dataDxfId="49">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ChangePercent" dataDxfId="50">
       <calculatedColumnFormula array="1">_FV(B2,"Change (%)",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Change" dataDxfId="48">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Change" dataDxfId="49">
       <calculatedColumnFormula array="1">_FV(B2,"Change")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="P/E" dataDxfId="47">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="P/E" dataDxfId="48">
       <calculatedColumnFormula array="1">_FV(B2,"P/E",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Beta" dataDxfId="46">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Beta" dataDxfId="47">
       <calculatedColumnFormula array="1">_FV(B2,"Beta")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="52WkHigh" dataDxfId="45">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="52WkHigh" dataDxfId="46">
       <calculatedColumnFormula array="1">_FV(B2,"52 week high",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="52WkLow" dataDxfId="44">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="52WkLow" dataDxfId="45">
       <calculatedColumnFormula array="1">_FV(B2,"52 week low",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="DayHigh" dataDxfId="43">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="DayHigh" dataDxfId="44">
       <calculatedColumnFormula array="1">_FV(B2,"High")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DayLow" dataDxfId="42">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DayLow" dataDxfId="43">
       <calculatedColumnFormula array="1">_FV(B2,"Low")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Open" dataDxfId="41">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Open" dataDxfId="42">
       <calculatedColumnFormula array="1">_FV(B2,"Open")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="PreviousClose" dataDxfId="40">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="PreviousClose" dataDxfId="41">
       <calculatedColumnFormula array="1">_FV(B2,"Previous close",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Volume" dataDxfId="39">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Volume" dataDxfId="40">
       <calculatedColumnFormula array="1">_FV(B2,"Volume")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="AverageVolume" dataDxfId="38">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="AverageVolume" dataDxfId="39">
       <calculatedColumnFormula array="1">_FV(B2,"Volume average",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="YearIncorported" dataDxfId="37">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="YearIncorported" dataDxfId="38">
       <calculatedColumnFormula array="1">_FV(B2,"Year incorporated",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Employees" dataDxfId="36">
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Employees" dataDxfId="37">
       <calculatedColumnFormula array="1">_FV(B2,"Employees")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Industry">
       <calculatedColumnFormula array="1">_FV(B2,"Industry")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="MarketCap" dataDxfId="35">
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="MarketCap" dataDxfId="36">
       <calculatedColumnFormula array="1">_FV(B2,"Market cap",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="SharesOutstanding" dataDxfId="34">
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="SharesOutstanding" dataDxfId="35">
       <calculatedColumnFormula array="1">_FV(B2,"Shares outstanding",TRUE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="50SMA"/>
@@ -9614,35 +9650,38 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}" name="tblHoldings" displayName="tblHoldings" ref="A1:M11" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32" tableBorderDxfId="31">
-  <autoFilter ref="A1:M11" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE3CE10F-629F-414E-93DE-8949C4E58E7D}" name="Symbol" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{40700DF4-EB97-4DB9-BA32-772C3F8E34CC}" name="StockName" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{BED1527E-0498-4FF1-8E69-ECDB2EB30C25}" name="TradeCurrency" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}" name="tblHoldings" displayName="tblHoldings" ref="A1:N11" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33" tableBorderDxfId="32">
+  <autoFilter ref="A1:N11" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{AE3CE10F-629F-414E-93DE-8949C4E58E7D}" name="Symbol" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{40700DF4-EB97-4DB9-BA32-772C3F8E34CC}" name="StockName" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{BED1527E-0498-4FF1-8E69-ECDB2EB30C25}" name="TradeCurrency" dataDxfId="29">
       <calculatedColumnFormula>_FV(B2,"Currency")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2218CAC2-8A57-48EA-B1D3-CD7E0BA08ECA}" name="TotalBought" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{77160EAF-769F-4559-B5AE-C08A0AC76566}" name="TotalSold" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{324BA50C-3A95-4946-A384-C4EF731BD7F3}" name="NetPosition" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{24A211AE-9FE1-4D72-98D4-96F240F7DCFD}" name="AvgCost" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{E1C8BF44-8957-447E-B3C1-A76A00A619B8}" name="AvgBuyCost" dataDxfId="23">
+    <tableColumn id="4" xr3:uid="{2218CAC2-8A57-48EA-B1D3-CD7E0BA08ECA}" name="TotalBought" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{77160EAF-769F-4559-B5AE-C08A0AC76566}" name="TotalSold" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{324BA50C-3A95-4946-A384-C4EF731BD7F3}" name="NetPosition" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{24A211AE-9FE1-4D72-98D4-96F240F7DCFD}" name="AvgCost" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{E1C8BF44-8957-447E-B3C1-A76A00A619B8}" name="AvgBuyCost" dataDxfId="24">
       <calculatedColumnFormula>F2*G2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{73ED87C5-FB66-49D5-B1EF-4BE32DC6D51F}" name="StockPrice" dataDxfId="22">
+    <tableColumn id="9" xr3:uid="{73ED87C5-FB66-49D5-B1EF-4BE32DC6D51F}" name="StockPrice" dataDxfId="23">
       <calculatedColumnFormula>_FV(B2,"Price")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{1E08B942-A194-43F5-A7DB-404EC54A5C02}" name="FXRate" dataDxfId="21">
+    <tableColumn id="10" xr3:uid="{1E08B942-A194-43F5-A7DB-404EC54A5C02}" name="FXRate" dataDxfId="22">
       <calculatedColumnFormula>Config!$C$1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{96D6E4C8-F5BD-4A3E-88A2-BF403C882136}" name="MarketValue" dataDxfId="20">
+    <tableColumn id="14" xr3:uid="{42171935-FB72-4173-A1EB-132DDE8201DD}" name="Column1" dataDxfId="0">
+      <calculatedColumnFormula array="1">_FV(B2,"Change (%)",TRUE)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{96D6E4C8-F5BD-4A3E-88A2-BF403C882136}" name="MarketValue" dataDxfId="21">
       <calculatedColumnFormula>F2*I2*J2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E928C781-D2C4-42A1-A053-38B541581BCB}" name="P&amp;L" dataDxfId="19">
-      <calculatedColumnFormula>K2-H2</calculatedColumnFormula>
+    <tableColumn id="12" xr3:uid="{E928C781-D2C4-42A1-A053-38B541581BCB}" name="P&amp;L" dataDxfId="20">
+      <calculatedColumnFormula>L2-H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{53BE744D-B35A-4E6B-8EA9-E422203F974E}" name="P&amp;LPercent" dataDxfId="18">
-      <calculatedColumnFormula>IF(H2=0,"",L2/H2)</calculatedColumnFormula>
+    <tableColumn id="13" xr3:uid="{53BE744D-B35A-4E6B-8EA9-E422203F974E}" name="P&amp;LPercent" dataDxfId="19">
+      <calculatedColumnFormula>IF(H2=0,"",M2/H2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
@@ -19252,7 +19291,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{989027A5-E4FB-4AA7-BEAE-7B9653141BA1}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="15.4"/>
   <cols>
     <col min="1" max="1" width="9.86328125" style="16" bestFit="1" customWidth="1"/>
@@ -19265,13 +19304,14 @@
     <col min="8" max="8" width="11.53125" style="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" style="16" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1328125" style="16" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.1328125" style="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.1328125" style="16"/>
+    <col min="11" max="11" width="7.6640625" style="41" customWidth="1"/>
+    <col min="12" max="12" width="12.1328125" style="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.1328125" style="16" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.1328125" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="13" t="s">
         <v>312</v>
       </c>
@@ -19302,17 +19342,20 @@
       <c r="J1" s="15" t="s">
         <v>318</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="K1" s="39" t="s">
+        <v>607</v>
+      </c>
+      <c r="L1" s="15" t="s">
         <v>319</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="M1" s="15" t="s">
         <v>320</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="N1" s="15" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:13" hidden="1">
+    <row r="2" spans="1:14" hidden="1">
       <c r="A2" s="17" t="s">
         <v>35</v>
       </c>
@@ -19347,20 +19390,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K2" s="20">
-        <f t="shared" ref="K2:K11" ca="1" si="3">F2*I2*J2</f>
+      <c r="K2" s="40" cm="1">
+        <f t="array" aca="1" ref="K2" ca="1">_FV(B2,"Change (%)",TRUE)</f>
+        <v>-1.8426000000000001E-2</v>
+      </c>
+      <c r="L2" s="20">
+        <f t="shared" ref="L2:L11" ca="1" si="3">F2*I2*J2</f>
         <v>2046.3652169999998</v>
       </c>
-      <c r="L2" s="20">
-        <f t="shared" ref="L2:L11" ca="1" si="4">K2-H2</f>
+      <c r="M2" s="20">
+        <f t="shared" ref="M2:M11" ca="1" si="4">L2-H2</f>
         <v>1741.2089669999998</v>
       </c>
-      <c r="M2" s="23">
-        <f t="shared" ref="M2:M11" ca="1" si="5">IF(H2=0,"",L2/H2)</f>
+      <c r="N2" s="23">
+        <f t="shared" ref="N2:N11" ca="1" si="5">IF(H2=0,"",M2/H2)</f>
         <v>5.7059587244239625</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:14">
       <c r="A3" s="17" t="s">
         <v>41</v>
       </c>
@@ -19395,20 +19442,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K3" s="20">
+      <c r="K3" s="40" cm="1">
+        <f t="array" aca="1" ref="K3" ca="1">_FV(B3,"Change (%)",TRUE)</f>
+        <v>-5.0654999999999999E-2</v>
+      </c>
+      <c r="L3" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>2674.373286</v>
       </c>
-      <c r="L3" s="20">
+      <c r="M3" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>-493.48671600000034</v>
       </c>
-      <c r="M3" s="23">
+      <c r="N3" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>-0.15577920605343729</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:14">
       <c r="A4" s="17" t="s">
         <v>60</v>
       </c>
@@ -19443,20 +19494,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K4" s="20">
+      <c r="K4" s="40" cm="1">
+        <f t="array" aca="1" ref="K4" ca="1">_FV(B4,"Change (%)",TRUE)</f>
+        <v>-3.7858000000000003E-2</v>
+      </c>
+      <c r="L4" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>5051.1659249999993</v>
       </c>
-      <c r="L4" s="20">
+      <c r="M4" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>1403.3666250000001</v>
       </c>
-      <c r="M4" s="23">
+      <c r="N4" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>0.38471596422533455</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:14">
       <c r="A5" s="17" t="s">
         <v>200</v>
       </c>
@@ -19491,20 +19546,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K5" s="20">
+      <c r="K5" s="40" cm="1">
+        <f t="array" aca="1" ref="K5" ca="1">_FV(B5,"Change (%)",TRUE)</f>
+        <v>6.2612000000000001E-2</v>
+      </c>
+      <c r="L5" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>2997.763704</v>
       </c>
-      <c r="L5" s="20">
+      <c r="M5" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>665.32370399999991</v>
       </c>
-      <c r="M5" s="23">
+      <c r="N5" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>0.28524793949683591</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:14">
       <c r="A6" s="17" t="s">
         <v>63</v>
       </c>
@@ -19539,20 +19598,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K6" s="20">
+      <c r="K6" s="40" cm="1">
+        <f t="array" aca="1" ref="K6" ca="1">_FV(B6,"Change (%)",TRUE)</f>
+        <v>-1.1568E-2</v>
+      </c>
+      <c r="L6" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>4544.0339879999992</v>
       </c>
-      <c r="L6" s="20">
+      <c r="M6" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>2684.5139879999992</v>
       </c>
-      <c r="M6" s="23">
+      <c r="N6" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>1.4436596476510064</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:14">
       <c r="A7" s="17" t="s">
         <v>70</v>
       </c>
@@ -19587,20 +19650,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K7" s="20">
+      <c r="K7" s="40" cm="1">
+        <f t="array" aca="1" ref="K7" ca="1">_FV(B7,"Change (%)",TRUE)</f>
+        <v>0.139596</v>
+      </c>
+      <c r="L7" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>2872.2704659999995</v>
       </c>
-      <c r="L7" s="20">
+      <c r="M7" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>798.18046699999923</v>
       </c>
-      <c r="M7" s="23">
+      <c r="N7" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>0.38483405608475679</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:14">
       <c r="A8" s="17" t="s">
         <v>64</v>
       </c>
@@ -19635,20 +19702,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K8" s="20">
+      <c r="K8" s="40" cm="1">
+        <f t="array" aca="1" ref="K8" ca="1">_FV(B8,"Change (%)",TRUE)</f>
+        <v>-4.5686999999999998E-2</v>
+      </c>
+      <c r="L8" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>5556.7390319999995</v>
       </c>
-      <c r="L8" s="20">
+      <c r="M8" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>702.46913200000017</v>
       </c>
-      <c r="M8" s="23">
+      <c r="N8" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>0.14471159339533227</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:14">
       <c r="A9" s="17" t="s">
         <v>76</v>
       </c>
@@ -19683,20 +19754,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K9" s="20">
+      <c r="K9" s="40" cm="1">
+        <f t="array" aca="1" ref="K9" ca="1">_FV(B9,"Change (%)",TRUE)</f>
+        <v>1.4733000000000001E-2</v>
+      </c>
+      <c r="L9" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>1014.3381039999999</v>
       </c>
-      <c r="L9" s="20">
+      <c r="M9" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>-78.891900000000078</v>
       </c>
-      <c r="M9" s="23">
+      <c r="N9" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>-7.2164045728112011E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:14">
       <c r="A10" s="17" t="s">
         <v>80</v>
       </c>
@@ -19731,20 +19806,24 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K10" s="20">
+      <c r="K10" s="40" cm="1">
+        <f t="array" aca="1" ref="K10" ca="1">_FV(B10,"Change (%)",TRUE)</f>
+        <v>0.130187</v>
+      </c>
+      <c r="L10" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>4598.5039619999998</v>
       </c>
-      <c r="L10" s="20">
+      <c r="M10" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>2088.6338259999993</v>
       </c>
-      <c r="M10" s="23">
+      <c r="N10" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>0.83216808552838961</v>
       </c>
     </row>
-    <row r="11" spans="1:13" hidden="1">
+    <row r="11" spans="1:14" hidden="1">
       <c r="A11" s="17" t="s">
         <v>32</v>
       </c>
@@ -19779,83 +19858,87 @@
         <f ca="1">Config!$C$1</f>
         <v>0.74229999999999996</v>
       </c>
-      <c r="K11" s="20">
+      <c r="K11" s="40" cm="1">
+        <f t="array" aca="1" ref="K11" ca="1">_FV(B11,"Change (%)",TRUE)</f>
+        <v>-1.4322999999999999E-2</v>
+      </c>
+      <c r="L11" s="20">
         <f t="shared" ca="1" si="3"/>
         <v>33203.078999999998</v>
       </c>
-      <c r="L11" s="20">
+      <c r="M11" s="20">
         <f t="shared" ca="1" si="4"/>
         <v>28203.078999999998</v>
       </c>
-      <c r="M11" s="23">
+      <c r="N11" s="23">
         <f t="shared" ca="1" si="5"/>
         <v>5.6406158</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A11">
-    <cfRule type="expression" dxfId="17" priority="16" stopIfTrue="1">
-      <formula>L2&gt;0</formula>
+    <cfRule type="expression" dxfId="18" priority="16" stopIfTrue="1">
+      <formula>M2&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="17" stopIfTrue="1">
-      <formula>L2&lt;0</formula>
+    <cfRule type="expression" dxfId="17" priority="17" stopIfTrue="1">
+      <formula>M2&lt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="18" stopIfTrue="1">
-      <formula>L2=0</formula>
+    <cfRule type="expression" dxfId="16" priority="18" stopIfTrue="1">
+      <formula>M2=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G11">
-    <cfRule type="cellIs" dxfId="14" priority="1" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="1" stopIfTrue="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="2" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="3" stopIfTrue="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H11">
-    <cfRule type="cellIs" dxfId="11" priority="4" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="4" stopIfTrue="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="5" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="5" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="6" stopIfTrue="1" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K11">
-    <cfRule type="cellIs" dxfId="8" priority="7" stopIfTrue="1" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="9" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="6" stopIfTrue="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L11">
-    <cfRule type="cellIs" dxfId="5" priority="10" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="7" stopIfTrue="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="11" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="8" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="12" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="9" stopIfTrue="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M11">
-    <cfRule type="cellIs" dxfId="2" priority="13" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="10" stopIfTrue="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="14" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="11" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="15" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="12" stopIfTrue="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N11">
+    <cfRule type="cellIs" dxfId="3" priority="13" stopIfTrue="1" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="14" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="15" stopIfTrue="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
fix tx import data type mismatch
</commit_message>
<xml_diff>
--- a/dashboard/trading_system.xlsx
+++ b/dashboard/trading_system.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\husainnatha\tradingsystem\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E6BAE3-93A2-479D-872B-B28774A4B832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F217D80-1AF7-44C0-A5C5-8ADB27BC18E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONTRIBUTIONS" sheetId="11" r:id="rId1"/>
@@ -3355,6 +3355,63 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -3741,63 +3798,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -10668,7 +10668,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F82495E7-9F34-4C1F-83EC-FA45D59FA2BD}" name="tblContributions" displayName="tblContributions" ref="A1:C2" totalsRowShown="0">
   <autoFilter ref="A1:C2" xr:uid="{F82495E7-9F34-4C1F-83EC-FA45D59FA2BD}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{EAE9033F-E950-4D8F-AC60-78CCDA7A0C9E}" name="DATE" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{EAE9033F-E950-4D8F-AC60-78CCDA7A0C9E}" name="DATE" dataDxfId="27"/>
     <tableColumn id="2" xr3:uid="{1D40F1FF-D66C-4703-9DEC-93C768793D8F}" name="AMMOUNT"/>
     <tableColumn id="3" xr3:uid="{49855D82-DE07-4257-837D-DD0BE41E988B}" name="Notes"/>
   </tableColumns>
@@ -10712,64 +10712,64 @@
   <tableColumns count="31">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="symbol"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="StockName"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="LastTradeTime" dataDxfId="43">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="LastTradeTime" dataDxfId="26">
       <calculatedColumnFormula array="1">_FV(B2,"Last trade time",TRUE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="TradeCurrency">
       <calculatedColumnFormula array="1">_FV(B2,"Currency")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="StockPrice" dataDxfId="42">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="StockPrice" dataDxfId="25">
       <calculatedColumnFormula array="1">_FV(B2,"Price")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ChangePercent" dataDxfId="41">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ChangePercent" dataDxfId="24">
       <calculatedColumnFormula array="1">_FV(B2,"Change (%)",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Change" dataDxfId="40">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Change" dataDxfId="23">
       <calculatedColumnFormula array="1">_FV(B2,"Change")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="P/E" dataDxfId="39">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="P/E" dataDxfId="22">
       <calculatedColumnFormula array="1">_FV(B2,"P/E",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Beta" dataDxfId="38">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Beta" dataDxfId="21">
       <calculatedColumnFormula array="1">_FV(B2,"Beta")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="52WkHigh" dataDxfId="37">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="52WkHigh" dataDxfId="20">
       <calculatedColumnFormula array="1">_FV(B2,"52 week high",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="52WkLow" dataDxfId="36">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="52WkLow" dataDxfId="19">
       <calculatedColumnFormula array="1">_FV(B2,"52 week low",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="DayHigh" dataDxfId="35">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="DayHigh" dataDxfId="18">
       <calculatedColumnFormula array="1">_FV(B2,"High")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DayLow" dataDxfId="34">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DayLow" dataDxfId="17">
       <calculatedColumnFormula array="1">_FV(B2,"Low")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Open" dataDxfId="33">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Open" dataDxfId="16">
       <calculatedColumnFormula array="1">_FV(B2,"Open")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="PreviousClose" dataDxfId="32">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="PreviousClose" dataDxfId="15">
       <calculatedColumnFormula array="1">_FV(B2,"Previous close",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Volume" dataDxfId="31">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Volume" dataDxfId="14">
       <calculatedColumnFormula array="1">_FV(B2,"Volume")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="AverageVolume" dataDxfId="30">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="AverageVolume" dataDxfId="13">
       <calculatedColumnFormula array="1">_FV(B2,"Volume average",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="YearIncorported" dataDxfId="29">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="YearIncorported" dataDxfId="12">
       <calculatedColumnFormula array="1">_FV(B2,"Year incorporated",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Employees" dataDxfId="28">
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Employees" dataDxfId="11">
       <calculatedColumnFormula array="1">_FV(B2,"Employees")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Industry">
       <calculatedColumnFormula array="1">_FV(B2,"Industry")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="MarketCap" dataDxfId="27">
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="MarketCap" dataDxfId="10">
       <calculatedColumnFormula array="1">_FV(B2,"Market cap",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="SharesOutstanding" dataDxfId="26">
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="SharesOutstanding" dataDxfId="9">
       <calculatedColumnFormula array="1">_FV(B2,"Shares outstanding",TRUE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="50SMA"/>
@@ -10787,37 +10787,37 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}" name="tblHoldings" displayName="tblHoldings" ref="A1:N10" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" tableBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}" name="tblHoldings" displayName="tblHoldings" ref="A1:N10" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43" tableBorderDxfId="42">
   <autoFilter ref="A1:N10" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{AE3CE10F-629F-414E-93DE-8949C4E58E7D}" name="Symbol" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{40700DF4-EB97-4DB9-BA32-772C3F8E34CC}" name="StockName" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{BED1527E-0498-4FF1-8E69-ECDB2EB30C25}" name="TradeCurrency" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{AE3CE10F-629F-414E-93DE-8949C4E58E7D}" name="Symbol" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{40700DF4-EB97-4DB9-BA32-772C3F8E34CC}" name="StockName" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{BED1527E-0498-4FF1-8E69-ECDB2EB30C25}" name="TradeCurrency" dataDxfId="39">
       <calculatedColumnFormula>_FV(B2,"Currency")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2218CAC2-8A57-48EA-B1D3-CD7E0BA08ECA}" name="TotalBought" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{77160EAF-769F-4559-B5AE-C08A0AC76566}" name="TotalSold" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{324BA50C-3A95-4946-A384-C4EF731BD7F3}" name="NetPosition" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{24A211AE-9FE1-4D72-98D4-96F240F7DCFD}" name="AvgCost" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{E1C8BF44-8957-447E-B3C1-A76A00A619B8}" name="AvgBuyCost" dataDxfId="15">
+    <tableColumn id="4" xr3:uid="{2218CAC2-8A57-48EA-B1D3-CD7E0BA08ECA}" name="TotalBought" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{77160EAF-769F-4559-B5AE-C08A0AC76566}" name="TotalSold" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{324BA50C-3A95-4946-A384-C4EF731BD7F3}" name="NetPosition" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{24A211AE-9FE1-4D72-98D4-96F240F7DCFD}" name="AvgCost" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{E1C8BF44-8957-447E-B3C1-A76A00A619B8}" name="AvgBuyCost" dataDxfId="34">
       <calculatedColumnFormula>F2*G2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{73ED87C5-FB66-49D5-B1EF-4BE32DC6D51F}" name="StockPrice" dataDxfId="14">
+    <tableColumn id="9" xr3:uid="{73ED87C5-FB66-49D5-B1EF-4BE32DC6D51F}" name="StockPrice" dataDxfId="33">
       <calculatedColumnFormula>_FV(B2,"Price")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{1E08B942-A194-43F5-A7DB-404EC54A5C02}" name="FXRate" dataDxfId="13">
+    <tableColumn id="10" xr3:uid="{1E08B942-A194-43F5-A7DB-404EC54A5C02}" name="FXRate" dataDxfId="32">
       <calculatedColumnFormula>Config!$C$1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{42171935-FB72-4173-A1EB-132DDE8201DD}" name="ChangePercent" dataDxfId="12">
+    <tableColumn id="14" xr3:uid="{42171935-FB72-4173-A1EB-132DDE8201DD}" name="ChangePercent" dataDxfId="31">
       <calculatedColumnFormula array="1">_FV(B2,"Change (%)",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{96D6E4C8-F5BD-4A3E-88A2-BF403C882136}" name="MarketValue" dataDxfId="11">
+    <tableColumn id="11" xr3:uid="{96D6E4C8-F5BD-4A3E-88A2-BF403C882136}" name="MarketValue" dataDxfId="30">
       <calculatedColumnFormula>F2*I2*J2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E928C781-D2C4-42A1-A053-38B541581BCB}" name="P&amp;L" dataDxfId="10">
+    <tableColumn id="12" xr3:uid="{E928C781-D2C4-42A1-A053-38B541581BCB}" name="P&amp;L" dataDxfId="29">
       <calculatedColumnFormula>L2-H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{53BE744D-B35A-4E6B-8EA9-E422203F974E}" name="P&amp;LPercent" dataDxfId="9">
+    <tableColumn id="13" xr3:uid="{53BE744D-B35A-4E6B-8EA9-E422203F974E}" name="P&amp;LPercent" dataDxfId="28">
       <calculatedColumnFormula>IF(H2=0,"",M2/H2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>

</xml_diff>

<commit_message>
create sector map intelligence using metadata
</commit_message>
<xml_diff>
--- a/dashboard/trading_system.xlsx
+++ b/dashboard/trading_system.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\husainnatha\projects\tradingsystem\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B57D685-92A1-493F-B164-8DF10649BB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E273DB22-C03B-4538-B641-3832B74ED6B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,6 +27,7 @@
     <sheet name="decision_engineering" sheetId="9" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -3343,6 +3344,63 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -3730,63 +3788,6 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4163,9 +4164,9 @@
     <v>13</v>
     <v>12.24</v>
     <v>10.99</v>
-    <v>0.83940000000000003</v>
-    <v>-0.01</v>
-    <v>-8.3330000000000003E-4</v>
+    <v>0.83819999999999995</v>
+    <v>0.02</v>
+    <v>1.6669999999999999E-3</v>
     <v>CAD</v>
     <v>Atrium Mortgage Investment Corporation is a Canada-based company. The Company is a non-bank provider of residential and commercial mortgages that lends in urban centers in Canada. Its objectives are to provide its shareholders with dividends and preserve shareholders equity by lending within conservative risk parameters. Its investment strategy is to invest in commercial and residential mortgages from borrowers whose financing needs are not being met by the larger financial institutions. It finances various types of properties, which include residential houses, small multi-family residential properties comprising six units or fewer, residential apartment buildings, commercial and storefront retail properties, as well as residential and commercial land development sites. It also provides construction financing and short-term bridge loans to real estate developers. The Company is managed by Canadian Mortgage Capital Corporation (CMCC).</v>
     <v>0</v>
@@ -4173,22 +4174,22 @@
     <v>NEOE</v>
     <v>NEOE</v>
     <v>20 Adelaide Street East, Suite 900, TORONTO, ON, M5C 2T6 CA</v>
-    <v>12</v>
+    <v>12.02</v>
     <v>Banking Services</v>
     <v>Stock</v>
-    <v>46192.764133865625</v>
+    <v>46192.830443599218</v>
     <v>11.97</v>
-    <v>578393883</v>
+    <v>579841073</v>
     <v>ATRIUM MORTGAGE INVESTMENT CORPORATION</v>
     <v>ATRIUM MORTGAGE INVESTMENT CORPORATION</v>
     <v>11.99</v>
-    <v>11.3941</v>
+    <v>11.422599999999999</v>
     <v>12</v>
-    <v>11.99</v>
+    <v>12.02</v>
     <v>48239690</v>
     <v>AI</v>
     <v>ATRIUM MORTGAGE INVESTMENT CORPORATION (NEOE:AI)</v>
-    <v>1612</v>
+    <v>7512</v>
     <v>98760</v>
     <v>2001</v>
   </rv>
@@ -4813,7 +4814,7 @@
     <v>23</v>
     <v>115.25</v>
     <v>36.884999999999998</v>
-    <v>0.97540000000000004</v>
+    <v>0.97750000000000004</v>
     <v>0.44</v>
     <v>7.3460000000000001E-3</v>
     <v>EUR</v>
@@ -4826,20 +4827,20 @@
     <v>61.04</v>
     <v>Automobiles &amp; Auto Parts</v>
     <v>Stock</v>
-    <v>46192.753472222219</v>
+    <v>46192.836805555555</v>
     <v>54</v>
     <v>59.98</v>
     <v>54471310000</v>
     <v>Bayerische Motoren Werke AG</v>
     <v>Bayerische Motoren Werke AG</v>
     <v>59.98</v>
-    <v>5.59</v>
+    <v>5.4359999999999999</v>
     <v>59.9</v>
     <v>60.34</v>
     <v>615810400</v>
     <v>BMW</v>
     <v>Bayerische Motoren Werke AG (XFRA:BMW)</v>
-    <v>7690</v>
+    <v>7694</v>
     <v>2134990</v>
     <v>1995</v>
   </rv>
@@ -4886,7 +4887,7 @@
     <v>CADENCE DESIGN SYSTEMS, INC.</v>
     <v>CADENCE DESIGN SYSTEMS, INC.</v>
     <v>391.1</v>
-    <v>90.953000000000003</v>
+    <v>90.437700000000007</v>
     <v>389.6</v>
     <v>387.39</v>
     <v>389</v>
@@ -6247,7 +6248,7 @@
     <v>XNAS</v>
     <v>2603 CHALLENGER TECH CT, STE 100, ORLANDO, FL, 32826-2716 US</v>
     <v>15.32</v>
-    <v>Office Equipment</v>
+    <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
     <v>46191.999875983594</v>
     <v>137</v>
@@ -6381,7 +6382,7 @@
     <v>MCDONALD'S CORPORATION</v>
     <v>MCDONALD'S CORPORATION</v>
     <v>284.38</v>
-    <v>22.965499999999999</v>
+    <v>23.3949</v>
     <v>283.82</v>
     <v>278.61</v>
     <v>279.33999999999997</v>
@@ -6490,9 +6491,9 @@
     <v>520.26</v>
     <v>1.2418</v>
     <v>9.64</v>
-    <v>-4.1929999999999997E-3</v>
+    <v>-4.0429999999999997E-3</v>
     <v>1.6983999999999999E-2</v>
-    <v>-2.42</v>
+    <v>-2.3336000000000001</v>
     <v>USD</v>
     <v>Meta Platforms, Inc. is building human connections, powered by artificial intelligence and immersive technologies. The Company's products enable people to connect and share with friends and family through mobile devices, personal computers, virtual reality (VR) and mixed reality (MR) headsets, augmented reality (AR), and wearables. It also helps people discover and learn about what is going on in the world around them, enabling people to share their experiences, ideas, photos, videos, and other content with audiences ranging from their closest family members and friends to the public at large. The Company's segments include Family of Apps (FoA) and Reality Labs (RL). FoA segment includes Facebook, Instagram, Messenger, WhatsApp and Threads. RL segment includes its virtual, augmented, and mixed reality related consumer hardware, software and content. Its product offerings in VR include its Meta Quest devices, as well as software and content available through the Meta Horizon Store.</v>
     <v>77986</v>
@@ -6510,10 +6511,10 @@
     <v>META PLATFORMS, INC.</v>
     <v>META PLATFORMS, INC.</v>
     <v>572.82000000000005</v>
-    <v>17.215599999999998</v>
+    <v>17.507999999999999</v>
     <v>567.58000000000004</v>
     <v>577.22</v>
-    <v>574.79999999999995</v>
+    <v>574.88639999999998</v>
     <v>2538423000</v>
     <v>META</v>
     <v>META PLATFORMS, INC. (XNAS:META)</v>
@@ -6743,7 +6744,7 @@
     <v>MICRON TECHNOLOGY, INC.</v>
     <v>MICRON TECHNOLOGY, INC.</v>
     <v>1108.0650000000001</v>
-    <v>53.537300000000002</v>
+    <v>49.250500000000002</v>
     <v>1043.19</v>
     <v>1133.99</v>
     <v>1151.95</v>
@@ -6839,7 +6840,7 @@
     <v>39.805</v>
     <v>Textiles &amp; Apparel</v>
     <v>Stock</v>
-    <v>46192.707638888889</v>
+    <v>46192.836805555555</v>
     <v>177</v>
     <v>39.215000000000003</v>
     <v>98149420000</v>
@@ -7071,7 +7072,7 @@
     <v>ON SEMICONDUCTOR CORPORATION</v>
     <v>ON SEMICONDUCTOR CORPORATION</v>
     <v>117.89</v>
-    <v>86.846599999999995</v>
+    <v>80.635300000000001</v>
     <v>112.92</v>
     <v>121.62</v>
     <v>121.85</v>
@@ -7830,7 +7831,7 @@
     <v>23</v>
     <v>269.35000000000002</v>
     <v>132.24</v>
-    <v>1.1264000000000001</v>
+    <v>1.1285000000000001</v>
     <v>-0.72</v>
     <v>-5.339E-3</v>
     <v>EUR</v>
@@ -7843,7 +7844,7 @@
     <v>136.72</v>
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
-    <v>46192.756585648145</v>
+    <v>46192.836805555555</v>
     <v>239</v>
     <v>132.24</v>
     <v>262224200000</v>
@@ -7856,7 +7857,7 @@
     <v>1228504000</v>
     <v>SAP</v>
     <v>SAP SE (XETR:SAP)</v>
-    <v>7123330</v>
+    <v>7123362</v>
     <v>3044800</v>
     <v>2014</v>
   </rv>
@@ -7935,7 +7936,7 @@
     <v>30</v>
     <v>1335</v>
     <v>771.66</v>
-    <v>0.36309999999999998</v>
+    <v>0.3639</v>
     <v>9.8000000000000007</v>
     <v>0</v>
     <v>1.2206999999999999E-2</v>
@@ -9029,18 +9030,15 @@
     <v>34</v>
     <v>0.76859999999999995</v>
     <v>0.72099999999999997</v>
-    <v>-1.7160000000000001E-3</v>
-    <v>-2.2669999999999999E-3</v>
+    <v>-1.585E-3</v>
+    <v>-2.0939999999999999E-3</v>
     <v>GBP</v>
     <v>USD</v>
-    <v>0.75960000000000005</v>
     <v>Currency Pair</v>
-    <v>46192.767094907409</v>
-    <v>0.75529999999999997</v>
+    <v>46192.882361111115</v>
     <v>US Dollar/UK Pound Sterling FX Cross Rate</v>
-    <v>0.75680000000000003</v>
     <v>0.7571</v>
-    <v>0.75529999999999997</v>
+    <v>0.75549999999999995</v>
     <v>USDGBP</v>
     <v>USD/GBP</v>
   </rv>
@@ -9495,12 +9493,9 @@
     <k n="Change (%)"/>
     <k n="Currency" t="s"/>
     <k n="From currency" t="s"/>
-    <k n="High"/>
     <k n="Instrument type" t="s"/>
     <k n="Last trade time"/>
-    <k n="Low"/>
     <k n="Name" t="s"/>
-    <k n="Open"/>
     <k n="Previous close"/>
     <k n="Price"/>
     <k n="Ticker symbol" t="s"/>
@@ -9913,7 +9908,7 @@
       <v t="s">ExchangeID</v>
       <v t="s">%ProviderInfo</v>
     </a>
-    <a count="27">
+    <a count="24">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -9931,9 +9926,6 @@
       <v t="s">Currency</v>
       <v t="s">From currency</v>
       <v t="s">Previous close</v>
-      <v t="s">Open</v>
-      <v t="s">High</v>
-      <v t="s">Low</v>
       <v t="s">52 week high</v>
       <v t="s">52 week low</v>
       <v t="s">Instrument type</v>
@@ -10291,10 +10283,7 @@
       <v>1</v>
     </spb>
     <spb s="22">
-      <v>17</v>
-      <v>17</v>
       <v>3</v>
-      <v>17</v>
       <v>17</v>
       <v>17</v>
       <v>5</v>
@@ -10565,10 +10554,7 @@
     <k n="`%ProviderInfo" t="spb"/>
   </s>
   <s>
-    <k n="Low" t="i"/>
-    <k n="High" t="i"/>
     <k n="Name" t="i"/>
-    <k n="Open" t="i"/>
     <k n="Price" t="i"/>
     <k n="Change" t="i"/>
     <k n="Change (%)" t="i"/>
@@ -10673,7 +10659,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F82495E7-9F34-4C1F-83EC-FA45D59FA2BD}" name="tblContributions" displayName="tblContributions" ref="A1:C2" totalsRowShown="0">
   <autoFilter ref="A1:C2" xr:uid="{F82495E7-9F34-4C1F-83EC-FA45D59FA2BD}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{EAE9033F-E950-4D8F-AC60-78CCDA7A0C9E}" name="DATE" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{EAE9033F-E950-4D8F-AC60-78CCDA7A0C9E}" name="DATE" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{1D40F1FF-D66C-4703-9DEC-93C768793D8F}" name="AMMOUNT"/>
     <tableColumn id="3" xr3:uid="{49855D82-DE07-4257-837D-DD0BE41E988B}" name="Notes"/>
   </tableColumns>
@@ -10717,64 +10703,64 @@
   <tableColumns count="31">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="symbol"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="StockName"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="LastTradeTime" dataDxfId="40">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="LastTradeTime" dataDxfId="23">
       <calculatedColumnFormula array="1">_FV(B2,"Last trade time",TRUE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="TradeCurrency">
       <calculatedColumnFormula array="1">_FV(B2,"Currency")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="StockPrice" dataDxfId="39">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="StockPrice" dataDxfId="22">
       <calculatedColumnFormula array="1">_FV(B2,"Price")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ChangePercent" dataDxfId="38">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ChangePercent" dataDxfId="21">
       <calculatedColumnFormula array="1">_FV(B2,"Change (%)",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Change" dataDxfId="37">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Change" dataDxfId="20">
       <calculatedColumnFormula array="1">_FV(B2,"Change")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="P/E" dataDxfId="36">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="P/E" dataDxfId="19">
       <calculatedColumnFormula array="1">_FV(B2,"P/E",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Beta" dataDxfId="35">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Beta" dataDxfId="18">
       <calculatedColumnFormula array="1">_FV(B2,"Beta")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="52WkHigh" dataDxfId="34">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="52WkHigh" dataDxfId="17">
       <calculatedColumnFormula array="1">_FV(B2,"52 week high",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="52WkLow" dataDxfId="33">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="52WkLow" dataDxfId="16">
       <calculatedColumnFormula array="1">_FV(B2,"52 week low",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="DayHigh" dataDxfId="32">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="DayHigh" dataDxfId="15">
       <calculatedColumnFormula array="1">_FV(B2,"High")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DayLow" dataDxfId="31">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DayLow" dataDxfId="14">
       <calculatedColumnFormula array="1">_FV(B2,"Low")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Open" dataDxfId="30">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Open" dataDxfId="13">
       <calculatedColumnFormula array="1">_FV(B2,"Open")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="PreviousClose" dataDxfId="29">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="PreviousClose" dataDxfId="12">
       <calculatedColumnFormula array="1">_FV(B2,"Previous close",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Volume" dataDxfId="28">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Volume" dataDxfId="11">
       <calculatedColumnFormula array="1">_FV(B2,"Volume")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="AverageVolume" dataDxfId="27">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="AverageVolume" dataDxfId="10">
       <calculatedColumnFormula array="1">_FV(B2,"Volume average",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="YearIncorported" dataDxfId="26">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="YearIncorported" dataDxfId="9">
       <calculatedColumnFormula array="1">_FV(B2,"Year incorporated",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Employees" dataDxfId="25">
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Employees" dataDxfId="8">
       <calculatedColumnFormula array="1">_FV(B2,"Employees")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Industry">
       <calculatedColumnFormula array="1">_FV(B2,"Industry")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="MarketCap" dataDxfId="24">
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="MarketCap" dataDxfId="7">
       <calculatedColumnFormula array="1">_FV(B2,"Market cap",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="SharesOutstanding" dataDxfId="23">
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="SharesOutstanding" dataDxfId="6">
       <calculatedColumnFormula array="1">_FV(B2,"Shares outstanding",TRUE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="50SMA"/>
@@ -10792,37 +10778,37 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}" name="tblHoldings" displayName="tblHoldings" ref="A1:N9" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21" tableBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}" name="tblHoldings" displayName="tblHoldings" ref="A1:N9" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40" tableBorderDxfId="39">
   <autoFilter ref="A1:N9" xr:uid="{D39CE96F-8D2C-4A60-A43A-B3602E27FDC2}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{AE3CE10F-629F-414E-93DE-8949C4E58E7D}" name="Symbol" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{40700DF4-EB97-4DB9-BA32-772C3F8E34CC}" name="StockName" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{BED1527E-0498-4FF1-8E69-ECDB2EB30C25}" name="TradeCurrency" dataDxfId="17">
+    <tableColumn id="1" xr3:uid="{AE3CE10F-629F-414E-93DE-8949C4E58E7D}" name="Symbol" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{40700DF4-EB97-4DB9-BA32-772C3F8E34CC}" name="StockName" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{BED1527E-0498-4FF1-8E69-ECDB2EB30C25}" name="TradeCurrency" dataDxfId="36">
       <calculatedColumnFormula>_FV(B2,"Currency")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2218CAC2-8A57-48EA-B1D3-CD7E0BA08ECA}" name="TotalBought" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{77160EAF-769F-4559-B5AE-C08A0AC76566}" name="TotalSold" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{324BA50C-3A95-4946-A384-C4EF731BD7F3}" name="NetPosition" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{24A211AE-9FE1-4D72-98D4-96F240F7DCFD}" name="AvgCost" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{E1C8BF44-8957-447E-B3C1-A76A00A619B8}" name="AvgBuyCost" dataDxfId="12">
+    <tableColumn id="4" xr3:uid="{2218CAC2-8A57-48EA-B1D3-CD7E0BA08ECA}" name="TotalBought" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{77160EAF-769F-4559-B5AE-C08A0AC76566}" name="TotalSold" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{324BA50C-3A95-4946-A384-C4EF731BD7F3}" name="NetPosition" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{24A211AE-9FE1-4D72-98D4-96F240F7DCFD}" name="AvgCost" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{E1C8BF44-8957-447E-B3C1-A76A00A619B8}" name="AvgBuyCost" dataDxfId="31">
       <calculatedColumnFormula>F2*G2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{73ED87C5-FB66-49D5-B1EF-4BE32DC6D51F}" name="StockPrice" dataDxfId="11">
+    <tableColumn id="9" xr3:uid="{73ED87C5-FB66-49D5-B1EF-4BE32DC6D51F}" name="StockPrice" dataDxfId="30">
       <calculatedColumnFormula>_FV(B2,"Price")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{1E08B942-A194-43F5-A7DB-404EC54A5C02}" name="FXRate" dataDxfId="10">
+    <tableColumn id="10" xr3:uid="{1E08B942-A194-43F5-A7DB-404EC54A5C02}" name="FXRate" dataDxfId="29">
       <calculatedColumnFormula>Config!$C$1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{42171935-FB72-4173-A1EB-132DDE8201DD}" name="ChangePercent" dataDxfId="9">
+    <tableColumn id="14" xr3:uid="{42171935-FB72-4173-A1EB-132DDE8201DD}" name="ChangePercent" dataDxfId="28">
       <calculatedColumnFormula array="1">_FV(B2,"Change (%)",TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{96D6E4C8-F5BD-4A3E-88A2-BF403C882136}" name="MarketValue" dataDxfId="8">
+    <tableColumn id="11" xr3:uid="{96D6E4C8-F5BD-4A3E-88A2-BF403C882136}" name="MarketValue" dataDxfId="27">
       <calculatedColumnFormula>F2*I2*J2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E928C781-D2C4-42A1-A053-38B541581BCB}" name="P&amp;L" dataDxfId="7">
+    <tableColumn id="12" xr3:uid="{E928C781-D2C4-42A1-A053-38B541581BCB}" name="P&amp;L" dataDxfId="26">
       <calculatedColumnFormula>L2-H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{53BE744D-B35A-4E6B-8EA9-E422203F974E}" name="P&amp;LPercent" dataDxfId="6">
+    <tableColumn id="13" xr3:uid="{53BE744D-B35A-4E6B-8EA9-E422203F974E}" name="P&amp;LPercent" dataDxfId="25">
       <calculatedColumnFormula>IF(H2=0,"",M2/H2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -14926,7 +14912,7 @@
       </c>
       <c r="C6" s="2">
         <f t="array" aca="1" ref="C6" ca="1">_FV(B6,"Last trade time",TRUE)</f>
-        <v>46192.764133865625</v>
+        <v>46192.830443599218</v>
       </c>
       <c r="D6" t="str">
         <f t="array" aca="1" ref="D6" ca="1">_FV(B6,"Currency")</f>
@@ -14934,23 +14920,23 @@
       </c>
       <c r="E6" s="3">
         <f t="array" aca="1" ref="E6" ca="1">_FV(B6,"Price")</f>
-        <v>11.99</v>
+        <v>12.02</v>
       </c>
       <c r="F6" s="4">
         <f t="array" aca="1" ref="F6" ca="1">_FV(B6,"Change (%)",TRUE)</f>
-        <v>-8.3330000000000003E-4</v>
+        <v>1.6669999999999999E-3</v>
       </c>
       <c r="G6" s="5">
         <f t="array" aca="1" ref="G6" ca="1">_FV(B6,"Change")</f>
-        <v>-0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H6" s="6">
         <f t="array" aca="1" ref="H6" ca="1">_FV(B6,"P/E",TRUE)</f>
-        <v>11.3941</v>
+        <v>11.422599999999999</v>
       </c>
       <c r="I6" s="6">
         <f t="array" aca="1" ref="I6" ca="1">_FV(B6,"Beta")</f>
-        <v>0.83940000000000003</v>
+        <v>0.83819999999999995</v>
       </c>
       <c r="J6" s="3">
         <f t="array" aca="1" ref="J6" ca="1">_FV(B6,"52 week high",TRUE)</f>
@@ -14962,7 +14948,7 @@
       </c>
       <c r="L6" s="3">
         <f t="array" aca="1" ref="L6" ca="1">_FV(B6,"High")</f>
-        <v>12</v>
+        <v>12.02</v>
       </c>
       <c r="M6" s="3">
         <f t="array" aca="1" ref="M6" ca="1">_FV(B6,"Low")</f>
@@ -14978,7 +14964,7 @@
       </c>
       <c r="P6" s="7">
         <f t="array" aca="1" ref="P6" ca="1">_FV(B6,"Volume")</f>
-        <v>1612</v>
+        <v>7512</v>
       </c>
       <c r="Q6" s="7">
         <f t="array" aca="1" ref="Q6" ca="1">_FV(B6,"Volume average",TRUE)</f>
@@ -14998,7 +14984,7 @@
       </c>
       <c r="U6" s="7">
         <f t="array" aca="1" ref="U6" ca="1">_FV(B6,"Market cap",TRUE)</f>
-        <v>578393883</v>
+        <v>579841073</v>
       </c>
       <c r="V6" s="7">
         <f t="array" aca="1" ref="V6" ca="1">_FV(B6,"Shares outstanding",TRUE)</f>
@@ -15982,7 +15968,7 @@
       </c>
       <c r="C18" s="2" cm="1">
         <f t="array" aca="1" ref="C18" ca="1">_FV(B18,"Last trade time",TRUE)</f>
-        <v>46192.753472222219</v>
+        <v>46192.836805555555</v>
       </c>
       <c r="D18" t="str" cm="1">
         <f t="array" aca="1" ref="D18" ca="1">_FV(B18,"Currency")</f>
@@ -16002,11 +15988,11 @@
       </c>
       <c r="H18" s="6" cm="1">
         <f t="array" aca="1" ref="H18" ca="1">_FV(B18,"P/E",TRUE)</f>
-        <v>5.59</v>
+        <v>5.4359999999999999</v>
       </c>
       <c r="I18" s="6" cm="1">
         <f t="array" aca="1" ref="I18" ca="1">_FV(B18,"Beta")</f>
-        <v>0.97540000000000004</v>
+        <v>0.97750000000000004</v>
       </c>
       <c r="J18" s="3" cm="1">
         <f t="array" aca="1" ref="J18" ca="1">_FV(B18,"52 week high",TRUE)</f>
@@ -16034,7 +16020,7 @@
       </c>
       <c r="P18" s="7" cm="1">
         <f t="array" aca="1" ref="P18" ca="1">_FV(B18,"Volume")</f>
-        <v>7690</v>
+        <v>7694</v>
       </c>
       <c r="Q18" s="7" cm="1">
         <f t="array" aca="1" ref="Q18" ca="1">_FV(B18,"Volume average",TRUE)</f>
@@ -16090,7 +16076,7 @@
       </c>
       <c r="H19" s="6" cm="1">
         <f t="array" aca="1" ref="H19" ca="1">_FV(B19,"P/E",TRUE)</f>
-        <v>90.953000000000003</v>
+        <v>90.437700000000007</v>
       </c>
       <c r="I19" s="6" cm="1">
         <f t="array" aca="1" ref="I19" ca="1">_FV(B19,"Beta")</f>
@@ -18426,7 +18412,7 @@
       </c>
       <c r="T45" t="str">
         <f t="array" aca="1" ref="T45" ca="1">_FV(B45,"Industry")</f>
-        <v>Office Equipment</v>
+        <v>Computers, Phones &amp; Household Electronics</v>
       </c>
       <c r="U45" s="7">
         <f t="array" aca="1" ref="U45" ca="1">_FV(B45,"Market cap",TRUE)</f>
@@ -18554,7 +18540,7 @@
       </c>
       <c r="H47" s="6" cm="1">
         <f t="array" aca="1" ref="H47" ca="1">_FV(B47,"P/E",TRUE)</f>
-        <v>22.965499999999999</v>
+        <v>23.3949</v>
       </c>
       <c r="I47" s="6" cm="1">
         <f t="array" aca="1" ref="I47" ca="1">_FV(B47,"Beta")</f>
@@ -18730,7 +18716,7 @@
       </c>
       <c r="H49" s="6">
         <f t="array" aca="1" ref="H49" ca="1">_FV(B49,"P/E",TRUE)</f>
-        <v>17.215599999999998</v>
+        <v>17.507999999999999</v>
       </c>
       <c r="I49" s="6">
         <f t="array" aca="1" ref="I49" ca="1">_FV(B49,"Beta")</f>
@@ -19082,7 +19068,7 @@
       </c>
       <c r="H53" s="6">
         <f t="array" aca="1" ref="H53" ca="1">_FV(B53,"P/E",TRUE)</f>
-        <v>53.537300000000002</v>
+        <v>49.250500000000002</v>
       </c>
       <c r="I53" s="6">
         <f t="array" aca="1" ref="I53" ca="1">_FV(B53,"Beta")</f>
@@ -19238,7 +19224,7 @@
       </c>
       <c r="C55" s="2" cm="1">
         <f t="array" aca="1" ref="C55" ca="1">_FV(B55,"Last trade time",TRUE)</f>
-        <v>46192.707638888889</v>
+        <v>46192.836805555555</v>
       </c>
       <c r="D55" t="str" cm="1">
         <f t="array" aca="1" ref="D55" ca="1">_FV(B55,"Currency")</f>
@@ -19610,7 +19596,7 @@
       </c>
       <c r="H59" s="6" cm="1">
         <f t="array" aca="1" ref="H59" ca="1">_FV(B59,"P/E",TRUE)</f>
-        <v>86.846599999999995</v>
+        <v>80.635300000000001</v>
       </c>
       <c r="I59" s="6" cm="1">
         <f t="array" aca="1" ref="I59" ca="1">_FV(B59,"Beta")</f>
@@ -20822,7 +20808,7 @@
       </c>
       <c r="C73" s="2" cm="1">
         <f t="array" aca="1" ref="C73" ca="1">_FV(B73,"Last trade time",TRUE)</f>
-        <v>46192.756585648145</v>
+        <v>46192.836805555555</v>
       </c>
       <c r="D73" t="str" cm="1">
         <f t="array" aca="1" ref="D73" ca="1">_FV(B73,"Currency")</f>
@@ -20846,7 +20832,7 @@
       </c>
       <c r="I73" s="6" cm="1">
         <f t="array" aca="1" ref="I73" ca="1">_FV(B73,"Beta")</f>
-        <v>1.1264000000000001</v>
+        <v>1.1285000000000001</v>
       </c>
       <c r="J73" s="3" cm="1">
         <f t="array" aca="1" ref="J73" ca="1">_FV(B73,"52 week high",TRUE)</f>
@@ -20874,7 +20860,7 @@
       </c>
       <c r="P73" s="7" cm="1">
         <f t="array" aca="1" ref="P73" ca="1">_FV(B73,"Volume")</f>
-        <v>7123330</v>
+        <v>7123362</v>
       </c>
       <c r="Q73" s="7" cm="1">
         <f t="array" aca="1" ref="Q73" ca="1">_FV(B73,"Volume average",TRUE)</f>
@@ -21022,7 +21008,7 @@
       </c>
       <c r="I75" s="6">
         <f t="array" aca="1" ref="I75" ca="1">_FV(B75,"Beta")</f>
-        <v>0.36309999999999998</v>
+        <v>0.3639</v>
       </c>
       <c r="J75" s="9">
         <f t="array" aca="1" ref="J75" ca="1">_FV(B75,"52 week high",TRUE)</f>
@@ -22945,7 +22931,7 @@
       </c>
       <c r="J2" s="47">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K2" s="48" cm="1">
         <f t="array" aca="1" ref="K2" ca="1">_FV(B2,"Change (%)",TRUE)</f>
@@ -22953,15 +22939,15 @@
       </c>
       <c r="L2" s="45">
         <f t="shared" ref="L2:L9" ca="1" si="2">F2*I2*J2</f>
-        <v>2615.8455960000001</v>
+        <v>2616.5382599999998</v>
       </c>
       <c r="M2" s="45">
         <f t="shared" ref="M2:M9" ca="1" si="3">L2-H2</f>
-        <v>-552.01440600000024</v>
+        <v>-551.32174200000054</v>
       </c>
       <c r="N2" s="48">
         <f t="shared" ref="N2:N9" ca="1" si="4">IF(H2=0,"",M2/H2)</f>
-        <v>-0.17425467212928944</v>
+        <v>-0.17403601852731132</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="24">
@@ -22997,7 +22983,7 @@
       </c>
       <c r="J3" s="47">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K3" s="48" cm="1">
         <f t="array" aca="1" ref="K3" ca="1">_FV(B3,"Change (%)",TRUE)</f>
@@ -23005,15 +22991,15 @@
       </c>
       <c r="L3" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>2864.4148259999997</v>
+        <v>2865.1733099999997</v>
       </c>
       <c r="M3" s="45">
         <f t="shared" ca="1" si="3"/>
-        <v>531.97482599999967</v>
+        <v>532.73330999999962</v>
       </c>
       <c r="N3" s="48">
         <f t="shared" ca="1" si="4"/>
-        <v>0.22807653187220236</v>
+        <v>0.22840172094459005</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="24">
@@ -23049,7 +23035,7 @@
       </c>
       <c r="J4" s="47">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K4" s="48" cm="1">
         <f t="array" aca="1" ref="K4" ca="1">_FV(B4,"Change (%)",TRUE)</f>
@@ -23057,15 +23043,15 @@
       </c>
       <c r="L4" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>4870.5067319999998</v>
+        <v>4871.7964199999997</v>
       </c>
       <c r="M4" s="45">
         <f t="shared" ca="1" si="3"/>
-        <v>3010.9867319999998</v>
+        <v>3012.2764199999997</v>
       </c>
       <c r="N4" s="48">
         <f t="shared" ca="1" si="4"/>
-        <v>1.6192279362416107</v>
+        <v>1.6199214958699018</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="24">
@@ -23101,7 +23087,7 @@
       </c>
       <c r="J5" s="47">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K5" s="48" cm="1">
         <f t="array" aca="1" ref="K5" ca="1">_FV(B5,"Change (%)",TRUE)</f>
@@ -23109,15 +23095,15 @@
       </c>
       <c r="L5" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>2761.7166850000003</v>
+        <v>2762.447975</v>
       </c>
       <c r="M5" s="45">
         <f t="shared" ca="1" si="3"/>
-        <v>687.62668600000006</v>
+        <v>688.35797599999978</v>
       </c>
       <c r="N5" s="48">
         <f t="shared" ca="1" si="4"/>
-        <v>0.33153174950534053</v>
+        <v>0.33188433304817244</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="24">
@@ -23153,7 +23139,7 @@
       </c>
       <c r="J6" s="47">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K6" s="48" cm="1">
         <f t="array" aca="1" ref="K6" ca="1">_FV(B6,"Change (%)",TRUE)</f>
@@ -23161,15 +23147,15 @@
       </c>
       <c r="L6" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>5444.8217459999996</v>
+        <v>5446.2635099999998</v>
       </c>
       <c r="M6" s="45">
         <f t="shared" ca="1" si="3"/>
-        <v>590.5518460000003</v>
+        <v>591.99361000000044</v>
       </c>
       <c r="N6" s="48">
         <f t="shared" ca="1" si="4"/>
-        <v>0.12165616213470132</v>
+        <v>0.12195317157787219</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="24">
@@ -23205,7 +23191,7 @@
       </c>
       <c r="J7" s="47">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K7" s="48" cm="1">
         <f t="array" aca="1" ref="K7" ca="1">_FV(B7,"Change (%)",TRUE)</f>
@@ -23213,15 +23199,15 @@
       </c>
       <c r="L7" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>915.96741599999996</v>
+        <v>916.20995999999991</v>
       </c>
       <c r="M7" s="45">
         <f t="shared" ca="1" si="3"/>
-        <v>-177.26258800000005</v>
+        <v>-177.0200440000001</v>
       </c>
       <c r="N7" s="48">
         <f t="shared" ca="1" si="4"/>
-        <v>-0.1621457400102605</v>
+        <v>-0.16192388001820712</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="24">
@@ -23257,7 +23243,7 @@
       </c>
       <c r="J8" s="47">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K8" s="48" cm="1">
         <f t="array" aca="1" ref="K8" ca="1">_FV(B8,"Change (%)",TRUE)</f>
@@ -23265,15 +23251,15 @@
       </c>
       <c r="L8" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>4092.8951700000002</v>
+        <v>4093.9789500000002</v>
       </c>
       <c r="M8" s="45">
         <f t="shared" ca="1" si="3"/>
-        <v>1583.0250339999998</v>
+        <v>1584.1088139999997</v>
       </c>
       <c r="N8" s="48">
         <f t="shared" ca="1" si="4"/>
-        <v>0.63071989713494858</v>
+        <v>0.63115170433662604</v>
       </c>
     </row>
     <row r="9" spans="1:14" hidden="1">
@@ -23309,7 +23295,7 @@
       </c>
       <c r="J9" s="20">
         <f ca="1">Config!$C$1</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
       <c r="K9" s="36" cm="1">
         <f t="array" aca="1" ref="K9" ca="1">_FV(B9,"Change (%)",TRUE)</f>
@@ -23317,15 +23303,15 @@
       </c>
       <c r="L9" s="18">
         <f t="shared" ca="1" si="2"/>
-        <v>30687.839</v>
+        <v>30695.964999999997</v>
       </c>
       <c r="M9" s="18">
         <f t="shared" ca="1" si="3"/>
-        <v>25687.839</v>
+        <v>25695.964999999997</v>
       </c>
       <c r="N9" s="21">
         <f t="shared" ca="1" si="4"/>
-        <v>5.1375678000000002</v>
+        <v>5.1391929999999997</v>
       </c>
     </row>
   </sheetData>
@@ -23372,7 +23358,7 @@
       </c>
       <c r="C1" s="3" cm="1">
         <f t="array" aca="1" ref="C1" ca="1">_FV(B1,"Price")</f>
-        <v>0.75529999999999997</v>
+        <v>0.75549999999999995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>